<commit_message>
Create project folder structure
</commit_message>
<xml_diff>
--- a/object-register.xlsx
+++ b/object-register.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\Subsea Line Data Health Checker\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\subsea-line-data-health-checker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60CC5A20-DD13-4C17-91CD-E283F1049098}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6076EE3-B26F-4A4C-8D9F-492967A307F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Objects" sheetId="1" r:id="rId1"/>

</xml_diff>